<commit_message>
Database Testing | JDBC Connection | Configuration
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SeleniumFramework\OrangeHRMProject\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6F5293-A757-4008-9D1F-91C4E7C204C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1F92E-DCAF-4D70-8E9F-22D0F14FF4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -34,23 +34,38 @@
     <t>password</t>
   </si>
   <si>
-    <t>admin</t>
+    <t>rootgly</t>
   </si>
   <si>
-    <t>admin123</t>
+    <t>rootgly1</t>
   </si>
   <si>
-    <t>admin1</t>
+    <t>F_society01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -73,13 +88,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -360,6 +378,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="20.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -373,16 +394,16 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -394,6 +415,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C33E9AE6-9E4B-47EB-9753-4DAA58E55552}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -405,10 +429,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Database Testing | JDBC Connection | Implemented
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SeleniumFramework\OrangeHRMProject\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1F92E-DCAF-4D70-8E9F-22D0F14FF4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF3136D-7CA1-4B23-8933-022A51EA31A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="inValidLoginData" sheetId="2" r:id="rId2"/>
+    <sheet name="emplVerification" sheetId="3" r:id="rId2"/>
+    <sheet name="inValidLoginData" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="8">
   <si>
     <t>username</t>
   </si>
@@ -41,6 +42,15 @@
   </si>
   <si>
     <t>F_society01</t>
+  </si>
+  <si>
+    <t>emp_id</t>
+  </si>
+  <si>
+    <t>emp_name</t>
+  </si>
+  <si>
+    <t>Pinku</t>
   </si>
 </sst>
 </file>
@@ -412,6 +422,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9DEAD32-4E6E-4946-9A06-41CF2C608524}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="9.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C33E9AE6-9E4B-47EB-9753-4DAA58E55552}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Minor change in pom.xml
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SeleniumFramework\OrangeHRMProject\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF3136D-7CA1-4B23-8933-022A51EA31A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79559EC-6C5A-49EA-B6AC-0C5CB2AE79E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +76,12 @@
     <font>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -417,6 +423,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>